<commit_message>
properties as valid header names
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionResults/Protocol_All_IWF-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionResults/Protocol_All_IWF-A4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionResults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BBB4932-4553-4E71-A5F3-BE6D7EAA7B47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C72DAC2-9DB5-4FFF-8C3B-481721D4315D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
   <si>
     <t>${l.lotNumber}</t>
   </si>
@@ -236,9 +236,6 @@
     <t>${t.get("Timekeeper")}</t>
   </si>
   <si>
-    <t>${t.get("Results.Controller")}</t>
-  </si>
-  <si>
     <t>${t.get("Referee1")}</t>
   </si>
   <si>
@@ -296,12 +293,6 @@
     <t>${r.resAthleteName}</t>
   </si>
   <si>
-    <t>${bestRankingTitle}</t>
-  </si>
-  <si>
-    <t>${l.bestLifterScore}</t>
-  </si>
-  <si>
     <t>${session.referee1AsTO} ${session.referee1AsTO.federationId}</t>
   </si>
   <si>
@@ -365,9 +356,6 @@
     <t>${session.technicalController3AsTO} ${session.technicalController3AsTO.federationId}</t>
   </si>
   <si>
-    <t>${t.get("Doctor")</t>
-  </si>
-  <si>
     <t>${session.doctorAsTO} ${session.doctorAsTO.federationId}</t>
   </si>
   <si>
@@ -377,19 +365,43 @@
     <t>${session.doctor3AsTO} ${session.doctor3AsTO.federationId}</t>
   </si>
   <si>
-    <t>${t.get("TO.Role.COMPETITION_SECRETARY")</t>
-  </si>
-  <si>
-    <t>${t.get("JuryPresident")</t>
-  </si>
-  <si>
     <t>${t.get("Jury.JuryMember")}</t>
   </si>
   <si>
-    <t>${t.get("ReserveReferee")}</t>
-  </si>
-  <si>
-    <t>${t.get("ReserveJury")}</t>
+    <t>${session.competitionSecretaryAsTO} ${session.competitionSecretaryAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.reserveJuryAsTO != null ? t.get("ReserveJury") : ""}</t>
+  </si>
+  <si>
+    <t>${session.competitionSecretary2AsTO} ${session.competitionSecretary2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${t.get("CompetitionSecretary")}</t>
+  </si>
+  <si>
+    <t>${t.get("JuryPresident")}</t>
+  </si>
+  <si>
+    <t>${session.doctorAsTO != null ? t.get("Doctor") : ""}</t>
+  </si>
+  <si>
+    <t>${session.doctor2AsTO != null ? t.get("Doctor") : ""}</t>
+  </si>
+  <si>
+    <t>${session.doctor3AsTO != null ? t.get("Doctor") : ""}</t>
+  </si>
+  <si>
+    <t>${session.marshal2AsTO != null ? t.get("Marshall") : ""}</t>
+  </si>
+  <si>
+    <t>${session.reserveAsTO != null ? t.get("ReserveReferee") : ""}</t>
+  </si>
+  <si>
+    <t>${session.technicalControllerAsTO != null ? t.get("TechnicalController") : ""}</t>
+  </si>
+  <si>
+    <t>${session.technicalController3AsTO != null ? t.get("TechnicalController") : ""}</t>
   </si>
 </sst>
 </file>
@@ -397,10 +409,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="165" formatCode="_ * #,##0_)\ _$_ ;_ * \(#,##0&quot;) &quot;_$_ ;_ * \-??_)\ _$_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
-    <numFmt numFmtId="167" formatCode="0;\(0\);\-"/>
-    <numFmt numFmtId="168" formatCode="0.000;;\-"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_)\ _$_ ;_ * \(#,##0&quot;) &quot;_$_ ;_ * \-??_)\ _$_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
+    <numFmt numFmtId="166" formatCode="0;\(0\);\-"/>
+    <numFmt numFmtId="167" formatCode="0.000;;\-"/>
   </numFmts>
   <fonts count="32" x14ac:knownFonts="1">
     <font>
@@ -682,7 +694,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -830,63 +842,6 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
         <color indexed="8"/>
       </right>
       <top style="thin">
@@ -1077,7 +1032,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1088,7 +1043,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1102,14 +1057,14 @@
     <xf numFmtId="1" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1126,10 +1081,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1159,34 +1114,13 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1197,297 +1131,279 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="29" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="29" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="30" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="14" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="30" fillId="14" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="11" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="11" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -1510,31 +1426,7 @@
     <cellStyle name="Titre de la feuille" xfId="16" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2014,222 +1906,195 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62"/>
-      <c r="B1" s="63"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="66"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
+      <c r="A1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
+      <c r="S1" s="110"/>
+      <c r="T1" s="110"/>
+      <c r="U1" s="110"/>
+      <c r="V1" s="110"/>
+      <c r="W1" s="110"/>
+      <c r="X1" s="110"/>
+      <c r="Y1" s="110"/>
+      <c r="Z1" s="110"/>
     </row>
     <row r="2" spans="1:28" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="68"/>
-      <c r="B2" s="69"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="74"/>
-      <c r="Q2" s="75"/>
-      <c r="R2" s="75"/>
-      <c r="S2" s="75"/>
-      <c r="T2" s="75"/>
-      <c r="U2" s="73"/>
-      <c r="V2" s="66"/>
-      <c r="W2" s="71"/>
-      <c r="X2" s="73"/>
-      <c r="Y2" s="73"/>
-      <c r="Z2" s="76"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="50"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="53"/>
+      <c r="R2" s="53"/>
+      <c r="S2" s="53"/>
+      <c r="T2" s="53"/>
+      <c r="U2" s="51"/>
+      <c r="V2" s="13"/>
+      <c r="X2" s="51"/>
+      <c r="Y2" s="51"/>
     </row>
     <row r="3" spans="1:28" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="71"/>
-      <c r="B3" s="77"/>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="65"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="78"/>
-      <c r="O3" s="78"/>
-      <c r="P3" s="78"/>
-      <c r="Q3" s="78"/>
-      <c r="R3" s="78"/>
-      <c r="S3" s="79"/>
-      <c r="T3" s="79"/>
-      <c r="U3" s="80"/>
-      <c r="V3" s="66"/>
-      <c r="W3" s="71"/>
-      <c r="X3" s="81"/>
-      <c r="Y3" s="81"/>
-      <c r="Z3" s="76"/>
+      <c r="B3" s="54"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="83"/>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="55"/>
+      <c r="T3" s="55"/>
+      <c r="U3" s="56"/>
+      <c r="V3" s="13"/>
+      <c r="X3" s="57"/>
+      <c r="Y3" s="57"/>
     </row>
     <row r="4" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="82" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="82"/>
-      <c r="C4" s="82"/>
-      <c r="D4" s="82"/>
-      <c r="E4" s="82"/>
-      <c r="F4" s="82"/>
-      <c r="G4" s="82"/>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82"/>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="82"/>
-      <c r="O4" s="82"/>
-      <c r="P4" s="82"/>
-      <c r="Q4" s="82"/>
-      <c r="R4" s="82"/>
-      <c r="S4" s="82"/>
-      <c r="T4" s="82"/>
-      <c r="U4" s="82"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="82"/>
-      <c r="X4" s="82"/>
-      <c r="Y4" s="82"/>
-      <c r="Z4" s="82"/>
+      <c r="A4" s="115" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="115"/>
+      <c r="C4" s="115"/>
+      <c r="D4" s="115"/>
+      <c r="E4" s="115"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="115"/>
+      <c r="I4" s="115"/>
+      <c r="J4" s="115"/>
+      <c r="K4" s="115"/>
+      <c r="L4" s="115"/>
+      <c r="M4" s="115"/>
+      <c r="N4" s="115"/>
+      <c r="O4" s="115"/>
+      <c r="P4" s="115"/>
+      <c r="Q4" s="115"/>
+      <c r="R4" s="115"/>
+      <c r="S4" s="115"/>
+      <c r="T4" s="115"/>
+      <c r="U4" s="115"/>
+      <c r="V4" s="115"/>
+      <c r="W4" s="115"/>
+      <c r="X4" s="115"/>
+      <c r="Y4" s="115"/>
+      <c r="Z4" s="115"/>
     </row>
     <row r="5" spans="1:28" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="102" t="s">
+      <c r="A6" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="122"/>
-      <c r="C6" s="49" t="s">
+      <c r="B6" s="85"/>
+      <c r="C6" s="95" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="101"/>
-      <c r="E6" s="49" t="s">
+      <c r="D6" s="96"/>
+      <c r="E6" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="101"/>
-      <c r="G6" s="50" t="s">
+      <c r="F6" s="96"/>
+      <c r="G6" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="50" t="s">
+      <c r="H6" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="108" t="s">
+      <c r="I6" s="101" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="109"/>
-      <c r="K6" s="50" t="s">
+      <c r="J6" s="102"/>
+      <c r="K6" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="51" t="s">
+      <c r="L6" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="52"/>
-      <c r="N6" s="52"/>
-      <c r="O6" s="52"/>
-      <c r="P6" s="52"/>
-      <c r="Q6" s="51" t="s">
+      <c r="M6" s="112"/>
+      <c r="N6" s="112"/>
+      <c r="O6" s="112"/>
+      <c r="P6" s="112"/>
+      <c r="Q6" s="111" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="52"/>
-      <c r="S6" s="52"/>
-      <c r="T6" s="52"/>
-      <c r="U6" s="52"/>
-      <c r="V6" s="52"/>
-      <c r="W6" s="53" t="s">
+      <c r="R6" s="112"/>
+      <c r="S6" s="112"/>
+      <c r="T6" s="112"/>
+      <c r="U6" s="112"/>
+      <c r="V6" s="112"/>
+      <c r="W6" s="113" t="s">
         <v>25</v>
       </c>
-      <c r="X6" s="54"/>
-      <c r="Y6" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="Z6" s="37"/>
+      <c r="X6" s="114"/>
+      <c r="Y6" s="122"/>
+      <c r="Z6" s="122"/>
       <c r="AB6"/>
     </row>
     <row r="7" spans="1:28" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="102"/>
-      <c r="B7" s="122"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="100"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="100"/>
-      <c r="G7" s="56"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="110"/>
-      <c r="J7" s="111"/>
-      <c r="K7" s="56"/>
-      <c r="L7" s="57">
+      <c r="A7" s="84"/>
+      <c r="B7" s="85"/>
+      <c r="C7" s="97"/>
+      <c r="D7" s="98"/>
+      <c r="E7" s="97"/>
+      <c r="F7" s="98"/>
+      <c r="G7" s="89"/>
+      <c r="H7" s="89"/>
+      <c r="I7" s="103"/>
+      <c r="J7" s="104"/>
+      <c r="K7" s="89"/>
+      <c r="L7" s="42">
         <v>1</v>
       </c>
-      <c r="M7" s="58">
+      <c r="M7" s="43">
         <v>2</v>
       </c>
-      <c r="N7" s="58">
+      <c r="N7" s="43">
         <v>3</v>
       </c>
-      <c r="O7" s="59" t="s">
-        <v>60</v>
-      </c>
-      <c r="P7" s="60" t="s">
+      <c r="O7" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="P7" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="Q7" s="58">
+      <c r="Q7" s="43">
         <v>1</v>
       </c>
-      <c r="R7" s="58">
+      <c r="R7" s="43">
         <v>2</v>
       </c>
-      <c r="S7" s="114">
+      <c r="S7" s="116">
         <v>3</v>
       </c>
-      <c r="T7" s="115"/>
-      <c r="U7" s="59" t="s">
-        <v>60</v>
-      </c>
-      <c r="V7" s="60" t="s">
+      <c r="T7" s="117"/>
+      <c r="U7" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="V7" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="W7" s="61" t="s">
+      <c r="W7" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="X7" s="60" t="s">
+      <c r="X7" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="Y7" s="38"/>
-      <c r="Z7" s="39"/>
+      <c r="Y7" s="122"/>
+      <c r="Z7" s="122"/>
     </row>
     <row r="8" spans="1:28" s="11" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="18"/>
@@ -2246,10 +2111,12 @@
       <c r="L8" s="18"/>
       <c r="M8" s="19"/>
       <c r="N8" s="20"/>
+      <c r="Y8" s="123"/>
+      <c r="Z8" s="123"/>
     </row>
     <row r="9" spans="1:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" s="22"/>
       <c r="C9" s="23"/>
@@ -2273,37 +2140,37 @@
       <c r="U9" s="23"/>
       <c r="V9" s="23"/>
       <c r="W9" s="23"/>
-      <c r="X9" s="23"/>
-      <c r="Y9" s="23"/>
-      <c r="Z9" s="34"/>
+      <c r="X9" s="127"/>
+      <c r="Y9" s="125"/>
+      <c r="Z9" s="126"/>
       <c r="AB9"/>
     </row>
     <row r="10" spans="1:28" s="11" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="43"/>
-      <c r="E10" s="104" t="s">
+      <c r="D10" s="36"/>
+      <c r="E10" s="120" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="105"/>
-      <c r="G10" s="44" t="s">
+      <c r="F10" s="121"/>
+      <c r="G10" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="H10" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="106" t="s">
+      <c r="I10" s="99" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="107"/>
-      <c r="K10" s="45" t="s">
+      <c r="J10" s="100"/>
+      <c r="K10" s="38" t="s">
         <v>15</v>
       </c>
       <c r="L10" s="10" t="s">
@@ -2318,8 +2185,8 @@
       <c r="O10" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="P10" s="46" t="s">
-        <v>57</v>
+      <c r="P10" s="39" t="s">
+        <v>54</v>
       </c>
       <c r="Q10" s="10" t="s">
         <v>11</v>
@@ -2327,26 +2194,24 @@
       <c r="R10" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="S10" s="116" t="s">
+      <c r="S10" s="118" t="s">
         <v>13</v>
       </c>
-      <c r="T10" s="117"/>
+      <c r="T10" s="119"/>
       <c r="U10" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="V10" s="46" t="s">
-        <v>58</v>
-      </c>
-      <c r="W10" s="47" t="s">
+      <c r="V10" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="W10" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="X10" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y10" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z10" s="41"/>
+      <c r="X10" s="41" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y10" s="124"/>
+      <c r="Z10" s="124"/>
     </row>
     <row r="11" spans="1:28" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11"/>
@@ -2368,7 +2233,7 @@
     </row>
     <row r="12" spans="1:28" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M12" s="17"/>
     </row>
@@ -2395,105 +2260,101 @@
       <c r="T13" s="28"/>
       <c r="U13" s="28"/>
       <c r="V13" s="28"/>
-      <c r="W13" s="113"/>
-      <c r="X13" s="113"/>
+      <c r="W13" s="28"/>
+      <c r="X13" s="28"/>
       <c r="Y13" s="28"/>
       <c r="Z13" s="28"/>
     </row>
     <row r="14" spans="1:28" s="33" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="120" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="121"/>
-      <c r="C14" s="124"/>
-      <c r="D14" s="123" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" s="120" t="s">
+      <c r="A14" s="92" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="93"/>
+      <c r="C14" s="94"/>
+      <c r="D14" s="71" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="92" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="94"/>
+      <c r="G14" s="71" t="s">
         <v>43</v>
-      </c>
-      <c r="F14" s="124"/>
-      <c r="G14" s="123" t="s">
-        <v>44</v>
       </c>
       <c r="H14" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="120" t="s">
-        <v>42</v>
-      </c>
-      <c r="J14" s="121"/>
-      <c r="K14" s="132" t="s">
-        <v>42</v>
-      </c>
-      <c r="L14" s="132"/>
-      <c r="M14" s="132"/>
-      <c r="N14" s="132"/>
-      <c r="O14" s="132"/>
-      <c r="P14" s="133"/>
+      <c r="I14" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="J14" s="93"/>
+      <c r="K14" s="76" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" s="76"/>
+      <c r="M14" s="76"/>
+      <c r="N14" s="76"/>
+      <c r="O14" s="76"/>
+      <c r="P14" s="30"/>
       <c r="Q14" s="29" t="s">
         <v>20</v>
       </c>
       <c r="R14" s="29"/>
       <c r="S14" s="32"/>
-      <c r="T14" s="131" t="s">
+      <c r="T14" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="U14" s="132"/>
+      <c r="U14" s="76"/>
       <c r="V14" s="30"/>
-      <c r="W14" s="138"/>
-      <c r="X14" s="139"/>
-      <c r="Y14" s="138"/>
-      <c r="Z14" s="139"/>
+      <c r="W14" s="81"/>
+      <c r="Y14" s="81"/>
       <c r="AB14" s="30"/>
     </row>
     <row r="15" spans="1:28" s="24" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="118" t="s">
+      <c r="A15" s="106" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="107"/>
+      <c r="C15" s="108"/>
+      <c r="D15" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="119"/>
-      <c r="C15" s="144"/>
-      <c r="D15" s="126" t="s">
+      <c r="E15" s="86" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="87"/>
+      <c r="G15" s="75" t="s">
+        <v>46</v>
+      </c>
+      <c r="H15" s="72" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" s="90" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="142" t="s">
-        <v>38</v>
-      </c>
-      <c r="F15" s="143"/>
-      <c r="G15" s="128" t="s">
+      <c r="J15" s="91"/>
+      <c r="K15" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="H15" s="125" t="s">
-        <v>46</v>
-      </c>
-      <c r="I15" s="130" t="s">
+      <c r="L15" s="74" t="s">
+        <v>47</v>
+      </c>
+      <c r="M15" s="79"/>
+      <c r="N15" s="79"/>
+      <c r="O15" s="79"/>
+      <c r="P15" s="80"/>
+      <c r="Q15" s="27" t="s">
         <v>36</v>
-      </c>
-      <c r="J15" s="129"/>
-      <c r="K15" s="127" t="s">
-        <v>48</v>
-      </c>
-      <c r="L15" s="127" t="s">
-        <v>48</v>
-      </c>
-      <c r="M15" s="136"/>
-      <c r="N15" s="136"/>
-      <c r="O15" s="136"/>
-      <c r="P15" s="137"/>
-      <c r="Q15" s="27" t="s">
-        <v>37</v>
       </c>
       <c r="R15" s="27"/>
       <c r="S15" s="26"/>
-      <c r="T15" s="134" t="s">
-        <v>39</v>
-      </c>
-      <c r="U15" s="135"/>
+      <c r="T15" s="77" t="s">
+        <v>38</v>
+      </c>
+      <c r="U15" s="78"/>
       <c r="V15" s="26"/>
-      <c r="W15" s="140"/>
-      <c r="X15" s="141"/>
-      <c r="Y15" s="140"/>
-      <c r="Z15" s="141"/>
+      <c r="W15" s="82"/>
+      <c r="Y15" s="82"/>
       <c r="AB15" s="26"/>
     </row>
     <row r="16" spans="1:28" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2501,9 +2362,9 @@
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
       <c r="K16" s="7"/>
       <c r="L16" s="6"/>
       <c r="M16" s="14"/>
@@ -2526,9 +2387,9 @@
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
       <c r="K17" s="7"/>
       <c r="L17" s="6"/>
       <c r="M17" s="14"/>
@@ -2546,240 +2407,259 @@
       <c r="AA17" s="6"/>
       <c r="AB17" s="6"/>
     </row>
-    <row r="18" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B18" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="78" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="78"/>
+        <v>30</v>
+      </c>
+      <c r="D18" s="83" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" s="83"/>
       <c r="F18" s="13"/>
       <c r="G18" s="13"/>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="60" t="s">
+        <v>83</v>
+      </c>
+      <c r="J18" s="105" t="s">
+        <v>66</v>
+      </c>
+      <c r="K18" s="105"/>
+      <c r="L18" s="105"/>
+      <c r="M18" s="105"/>
+      <c r="N18" s="105"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="R18" s="5"/>
+      <c r="S18" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="T18"/>
+      <c r="U18" s="58" t="s">
+        <v>52</v>
+      </c>
+      <c r="V18" s="15"/>
+      <c r="W18" s="58"/>
+      <c r="X18"/>
+      <c r="AA18"/>
+    </row>
+    <row r="19" spans="1:28" s="61" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="J18" s="103" t="s">
-        <v>69</v>
-      </c>
-      <c r="K18" s="103"/>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="103"/>
-      <c r="S18" s="112" t="s">
-        <v>77</v>
-      </c>
-      <c r="U18" s="84" t="s">
-        <v>55</v>
-      </c>
-      <c r="V18" s="85"/>
-      <c r="W18" s="84"/>
-      <c r="Y18" s="64"/>
-      <c r="Z18" s="76"/>
-      <c r="AB18" s="64"/>
-    </row>
-    <row r="19" spans="1:28" s="88" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="78" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="78"/>
+      <c r="D19" s="83" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="83"/>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
-      <c r="H19" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J19" s="103" t="s">
-        <v>70</v>
-      </c>
-      <c r="K19" s="103"/>
-      <c r="L19" s="103"/>
-      <c r="M19" s="103"/>
-      <c r="N19" s="103"/>
-      <c r="S19" s="112" t="s">
-        <v>78</v>
-      </c>
-      <c r="T19" s="87"/>
-      <c r="U19" s="84" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z19" s="91"/>
-    </row>
-    <row r="20" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H19" s="60" t="s">
+        <v>83</v>
+      </c>
+      <c r="J19" s="105" t="s">
+        <v>67</v>
+      </c>
+      <c r="K19" s="105"/>
+      <c r="L19" s="105"/>
+      <c r="M19" s="105"/>
+      <c r="N19" s="105"/>
+      <c r="S19" s="60" t="s">
+        <v>72</v>
+      </c>
+      <c r="T19" s="60"/>
+      <c r="U19" s="58" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z19" s="64"/>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B20" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="78" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="78"/>
+        <v>31</v>
+      </c>
+      <c r="D20" s="83" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="83"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
-      <c r="H20" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J20" s="103" t="s">
-        <v>71</v>
-      </c>
-      <c r="K20" s="103"/>
-      <c r="L20" s="103"/>
-      <c r="M20" s="103"/>
-      <c r="N20" s="103"/>
-      <c r="S20" s="112" t="s">
+      <c r="H20" s="60" t="s">
+        <v>84</v>
+      </c>
+      <c r="J20" s="105" t="s">
+        <v>68</v>
+      </c>
+      <c r="K20" s="105"/>
+      <c r="L20" s="105"/>
+      <c r="M20" s="105"/>
+      <c r="N20" s="105"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="60" t="s">
+        <v>72</v>
+      </c>
+      <c r="U20" s="58" t="s">
+        <v>62</v>
+      </c>
+      <c r="V20" s="14"/>
+      <c r="W20" s="1"/>
+      <c r="X20"/>
+      <c r="Z20" s="4"/>
+      <c r="AB20"/>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B21" s="60" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="83"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="65"/>
+      <c r="J21" s="68"/>
+      <c r="K21" s="68"/>
+      <c r="L21" s="68"/>
+      <c r="M21" s="68"/>
+      <c r="N21"/>
+      <c r="O21"/>
+      <c r="P21"/>
+      <c r="R21" s="5"/>
+      <c r="S21" s="60" t="s">
+        <v>72</v>
+      </c>
+      <c r="U21" s="58" t="s">
+        <v>63</v>
+      </c>
+      <c r="V21" s="14"/>
+      <c r="W21" s="58"/>
+      <c r="X21"/>
+      <c r="Z21" s="1"/>
+      <c r="AB21"/>
+    </row>
+    <row r="22" spans="1:28" s="61" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="14"/>
+      <c r="D22" s="63"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="70"/>
+      <c r="G22" s="70"/>
+      <c r="H22" s="60" t="s">
+        <v>76</v>
+      </c>
+      <c r="J22" s="105" t="s">
+        <v>73</v>
+      </c>
+      <c r="K22" s="105"/>
+      <c r="L22" s="105"/>
+      <c r="M22" s="105"/>
+      <c r="N22" s="105"/>
+      <c r="S22" s="60" t="s">
+        <v>72</v>
+      </c>
+      <c r="U22" s="58" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z22" s="64"/>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B23" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="83" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="83"/>
+      <c r="F23" s="70"/>
+      <c r="G23" s="70"/>
+      <c r="H23" s="60" t="s">
+        <v>76</v>
+      </c>
+      <c r="J23" s="105" t="s">
+        <v>75</v>
+      </c>
+      <c r="K23" s="105"/>
+      <c r="L23" s="105"/>
+      <c r="M23" s="105"/>
+      <c r="N23" s="105"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="R23" s="5"/>
+      <c r="S23" s="60" t="s">
+        <v>74</v>
+      </c>
+      <c r="U23" s="83" t="s">
+        <v>65</v>
+      </c>
+      <c r="V23" s="83"/>
+      <c r="W23" s="83"/>
+      <c r="X23" s="83"/>
+      <c r="Y23" s="83"/>
+      <c r="Z23" s="83"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+    </row>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B24" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D24" s="83" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="83"/>
+      <c r="H24" s="5"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="R24"/>
+      <c r="X24"/>
+      <c r="Y24"/>
+      <c r="Z24" s="67"/>
+      <c r="AA24"/>
+      <c r="AB24"/>
+    </row>
+    <row r="25" spans="1:28" s="61" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="63"/>
+      <c r="E25" s="59"/>
+      <c r="F25" s="70"/>
+      <c r="G25" s="70"/>
+      <c r="H25" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="T20" s="64"/>
-      <c r="U20" s="84" t="s">
-        <v>65</v>
-      </c>
-      <c r="V20" s="83"/>
-      <c r="W20" s="64"/>
-      <c r="Y20" s="64"/>
-      <c r="Z20" s="95"/>
-      <c r="AA20" s="64"/>
-    </row>
-    <row r="21" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="14" t="s">
+      <c r="J25" s="105" t="s">
+        <v>69</v>
+      </c>
+      <c r="K25" s="105"/>
+      <c r="L25" s="105"/>
+      <c r="M25" s="105"/>
+      <c r="N25" s="105"/>
+      <c r="O25" s="59"/>
+      <c r="V25" s="59"/>
+      <c r="W25" s="59"/>
+      <c r="Z25" s="64"/>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B26" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="83" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="83"/>
+      <c r="F26" s="70"/>
+      <c r="G26" s="70"/>
+      <c r="H26" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="78" t="s">
-        <v>56</v>
-      </c>
-      <c r="E21" s="78"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="66"/>
-      <c r="H21" s="66"/>
-      <c r="J21" s="97"/>
-      <c r="K21" s="97"/>
-      <c r="L21" s="97"/>
-      <c r="M21" s="97"/>
-      <c r="S21" s="112" t="s">
-        <v>78</v>
-      </c>
-      <c r="T21" s="64"/>
-      <c r="U21" s="84" t="s">
-        <v>66</v>
-      </c>
-      <c r="V21" s="83"/>
-      <c r="W21" s="84"/>
-      <c r="Y21" s="64"/>
-      <c r="Z21" s="64"/>
-      <c r="AA21" s="64"/>
-    </row>
-    <row r="22" spans="1:28" s="88" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="14"/>
-      <c r="D22" s="90"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="112"/>
-      <c r="G22" s="112"/>
-      <c r="H22" s="112" t="s">
-        <v>76</v>
-      </c>
-      <c r="J22" s="103" t="s">
-        <v>73</v>
-      </c>
-      <c r="K22" s="103"/>
-      <c r="L22" s="103"/>
-      <c r="M22" s="103"/>
-      <c r="N22" s="103"/>
-      <c r="S22" s="112" t="s">
-        <v>78</v>
-      </c>
-      <c r="U22" s="84" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z22" s="91"/>
-    </row>
-    <row r="23" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="66" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="78" t="s">
-        <v>62</v>
-      </c>
-      <c r="E23" s="78"/>
-      <c r="F23" s="112"/>
-      <c r="G23" s="112"/>
-      <c r="H23" s="112" t="s">
-        <v>76</v>
-      </c>
-      <c r="J23" s="103" t="s">
-        <v>74</v>
-      </c>
-      <c r="K23" s="103"/>
-      <c r="L23" s="103"/>
-      <c r="M23" s="103"/>
-      <c r="N23" s="103"/>
-      <c r="S23" s="112" t="s">
-        <v>80</v>
-      </c>
-      <c r="T23" s="64"/>
-      <c r="U23" s="78" t="s">
-        <v>68</v>
-      </c>
-      <c r="V23" s="78"/>
-      <c r="W23" s="78"/>
-      <c r="X23" s="78"/>
-      <c r="Y23" s="78"/>
-      <c r="Z23" s="78"/>
-    </row>
-    <row r="24" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="66" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="78" t="s">
-        <v>63</v>
-      </c>
-      <c r="E24" s="78"/>
-      <c r="S24" s="64"/>
-      <c r="T24" s="64"/>
-      <c r="U24" s="64"/>
-      <c r="V24" s="64"/>
-      <c r="Z24" s="96"/>
-    </row>
-    <row r="25" spans="1:28" s="88" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D25" s="90"/>
-      <c r="E25" s="86"/>
-      <c r="F25" s="112"/>
-      <c r="G25" s="112"/>
-      <c r="H25" s="112" t="s">
-        <v>72</v>
-      </c>
-      <c r="J25" s="103" t="s">
-        <v>73</v>
-      </c>
-      <c r="K25" s="103"/>
-      <c r="L25" s="103"/>
-      <c r="M25" s="103"/>
-      <c r="N25" s="103"/>
-      <c r="O25" s="86"/>
-      <c r="V25" s="86"/>
-      <c r="W25" s="86"/>
-      <c r="Z25" s="91"/>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B26" s="66" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="78" t="s">
-        <v>54</v>
-      </c>
-      <c r="E26" s="78"/>
-      <c r="F26" s="112"/>
-      <c r="G26" s="112"/>
-      <c r="H26" s="112" t="s">
-        <v>72</v>
-      </c>
-      <c r="I26" s="71"/>
-      <c r="J26" s="103" t="s">
-        <v>74</v>
-      </c>
-      <c r="K26" s="103"/>
-      <c r="L26" s="103"/>
-      <c r="M26" s="103"/>
-      <c r="N26" s="103"/>
+      <c r="J26" s="105" t="s">
+        <v>70</v>
+      </c>
+      <c r="K26" s="105"/>
+      <c r="L26" s="105"/>
+      <c r="M26" s="105"/>
+      <c r="N26" s="105"/>
       <c r="P26"/>
       <c r="Q26" s="3"/>
       <c r="R26" s="1"/>
@@ -2788,312 +2668,176 @@
       <c r="X26" s="4"/>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="F27" s="112"/>
-      <c r="G27" s="112"/>
-      <c r="H27" s="112" t="s">
-        <v>72</v>
-      </c>
-      <c r="I27" s="71"/>
-      <c r="J27" s="103" t="s">
-        <v>75</v>
-      </c>
-      <c r="K27" s="103"/>
-      <c r="L27" s="103"/>
-      <c r="M27" s="103"/>
-      <c r="N27" s="103"/>
+      <c r="F27" s="70"/>
+      <c r="G27" s="70"/>
+      <c r="H27" s="60" t="s">
+        <v>80</v>
+      </c>
+      <c r="J27" s="105" t="s">
+        <v>71</v>
+      </c>
+      <c r="K27" s="105"/>
+      <c r="L27" s="105"/>
+      <c r="M27" s="105"/>
+      <c r="N27" s="105"/>
       <c r="Y27" s="4"/>
     </row>
-    <row r="28" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="64"/>
-      <c r="I28" s="64"/>
-      <c r="J28" s="64"/>
-      <c r="K28" s="64"/>
-      <c r="L28" s="65"/>
-      <c r="M28" s="64"/>
-      <c r="N28" s="64"/>
-      <c r="O28" s="64"/>
-      <c r="P28" s="64"/>
-      <c r="R28" s="76"/>
-      <c r="S28" s="64"/>
-      <c r="T28" s="64"/>
-      <c r="U28" s="64"/>
-      <c r="V28" s="64"/>
-      <c r="X28" s="64"/>
-      <c r="Y28" s="95"/>
-      <c r="Z28" s="76"/>
-      <c r="AA28" s="64"/>
-      <c r="AB28" s="64"/>
-    </row>
-    <row r="29" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="64"/>
-      <c r="I29" s="64"/>
-      <c r="J29" s="64"/>
-      <c r="K29" s="64"/>
-      <c r="L29" s="65"/>
-      <c r="M29" s="64"/>
-      <c r="N29" s="64"/>
-      <c r="O29" s="64"/>
-      <c r="P29" s="64"/>
-      <c r="R29" s="76"/>
-      <c r="S29" s="64"/>
-      <c r="T29" s="64"/>
-      <c r="U29" s="64"/>
-      <c r="V29" s="64"/>
-      <c r="X29" s="64"/>
-      <c r="Y29" s="95"/>
-      <c r="Z29" s="76"/>
-      <c r="AA29" s="64"/>
-      <c r="AB29" s="64"/>
-    </row>
-    <row r="30" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="64"/>
-      <c r="I30" s="64"/>
-      <c r="J30" s="64"/>
-      <c r="K30" s="64"/>
-      <c r="L30" s="65"/>
-      <c r="M30" s="64"/>
-      <c r="N30" s="64"/>
-      <c r="O30" s="64"/>
-      <c r="P30" s="64"/>
-      <c r="R30" s="76"/>
-      <c r="S30" s="64"/>
-      <c r="T30" s="64"/>
-      <c r="U30" s="64"/>
-      <c r="V30" s="64"/>
-      <c r="X30" s="64"/>
-      <c r="Y30" s="95"/>
-      <c r="Z30" s="76"/>
-      <c r="AA30" s="64"/>
-      <c r="AB30" s="64"/>
-    </row>
-    <row r="31" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="64"/>
-      <c r="I31" s="64"/>
-      <c r="J31" s="64"/>
-      <c r="K31" s="64"/>
-      <c r="L31" s="65"/>
-      <c r="M31" s="64"/>
-      <c r="N31" s="64"/>
-      <c r="O31" s="64"/>
-      <c r="P31" s="64"/>
-      <c r="R31" s="76"/>
-      <c r="S31" s="64"/>
-      <c r="T31" s="64"/>
-      <c r="U31" s="64"/>
-      <c r="V31" s="64"/>
-      <c r="X31" s="64"/>
-      <c r="Y31" s="95"/>
-      <c r="Z31" s="76"/>
-      <c r="AA31" s="64"/>
-      <c r="AB31" s="64"/>
-    </row>
-    <row r="32" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="64"/>
-      <c r="E32" s="98"/>
-      <c r="F32" s="98"/>
-      <c r="G32" s="98"/>
-      <c r="H32" s="98"/>
-      <c r="I32" s="64"/>
-      <c r="J32" s="64"/>
-      <c r="K32" s="64"/>
-      <c r="L32" s="65"/>
-      <c r="M32" s="64"/>
-      <c r="N32" s="64"/>
-      <c r="O32" s="64"/>
-      <c r="P32" s="64"/>
-      <c r="R32" s="76"/>
-      <c r="S32" s="64"/>
-      <c r="T32" s="64"/>
-      <c r="U32" s="64"/>
-      <c r="V32" s="64"/>
-      <c r="X32" s="64"/>
-      <c r="Y32" s="95"/>
-      <c r="Z32" s="76"/>
-      <c r="AA32" s="64"/>
-      <c r="AB32" s="64"/>
-    </row>
-    <row r="33" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="64"/>
-      <c r="I33" s="64"/>
-      <c r="J33" s="64"/>
-      <c r="K33" s="64"/>
-      <c r="L33" s="65"/>
-      <c r="M33" s="64"/>
-      <c r="N33" s="64"/>
-      <c r="O33" s="64"/>
-      <c r="P33" s="64"/>
-      <c r="R33" s="76"/>
-      <c r="S33" s="64"/>
-      <c r="T33" s="64"/>
-      <c r="U33" s="64"/>
-      <c r="V33" s="64"/>
-      <c r="X33" s="64"/>
-      <c r="Y33" s="95"/>
-      <c r="Z33" s="76"/>
-      <c r="AA33" s="64"/>
-      <c r="AB33" s="64"/>
-    </row>
-    <row r="34" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="64"/>
-      <c r="I34" s="64"/>
-      <c r="J34" s="64"/>
-      <c r="K34" s="64"/>
-      <c r="L34" s="65"/>
-      <c r="M34" s="64"/>
-      <c r="N34" s="64"/>
-      <c r="O34" s="64"/>
-      <c r="P34" s="64"/>
-      <c r="R34" s="76"/>
-      <c r="S34" s="64"/>
-      <c r="T34" s="64"/>
-      <c r="U34" s="64"/>
-      <c r="V34" s="64"/>
-      <c r="X34" s="64"/>
-      <c r="Y34" s="95"/>
-      <c r="Z34" s="76"/>
-      <c r="AA34" s="64"/>
-      <c r="AB34" s="64"/>
-    </row>
-    <row r="35" spans="1:28" s="71" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="64"/>
-      <c r="B35" s="83"/>
-      <c r="C35" s="84"/>
-      <c r="D35" s="84"/>
-      <c r="E35" s="64"/>
-      <c r="K35" s="64"/>
-      <c r="L35" s="64"/>
-      <c r="M35" s="64"/>
-      <c r="N35" s="64"/>
-      <c r="O35" s="84"/>
-      <c r="P35" s="64"/>
-      <c r="Q35" s="64"/>
-      <c r="R35" s="64"/>
-      <c r="U35" s="64"/>
-      <c r="V35" s="64"/>
-      <c r="W35" s="84"/>
-      <c r="Y35" s="64"/>
-      <c r="Z35" s="76"/>
-      <c r="AB35" s="64"/>
-    </row>
-    <row r="36" spans="1:28" s="88" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A36" s="86"/>
-      <c r="B36" s="87"/>
-      <c r="F36" s="89"/>
-      <c r="G36" s="89"/>
-      <c r="H36" s="89"/>
-      <c r="I36" s="90"/>
-      <c r="J36" s="90"/>
-      <c r="L36" s="86"/>
-      <c r="N36" s="89"/>
-      <c r="U36" s="86"/>
-      <c r="Z36" s="91"/>
-    </row>
-    <row r="37" spans="1:28" s="71" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="64"/>
-      <c r="B37" s="92"/>
-      <c r="E37" s="64"/>
-      <c r="F37" s="93"/>
-      <c r="G37" s="93"/>
-      <c r="H37" s="93"/>
-      <c r="I37" s="94"/>
-      <c r="J37" s="94"/>
-      <c r="K37" s="64"/>
-      <c r="L37" s="64"/>
-      <c r="M37" s="99"/>
-      <c r="N37" s="99"/>
-      <c r="O37" s="64"/>
-      <c r="Q37" s="64"/>
-      <c r="R37" s="95"/>
-      <c r="S37" s="64"/>
-      <c r="T37" s="64"/>
-      <c r="U37" s="64"/>
-      <c r="V37" s="64"/>
-      <c r="X37" s="64"/>
-      <c r="Y37" s="64"/>
-      <c r="Z37" s="95"/>
-      <c r="AA37" s="64"/>
-    </row>
-    <row r="38" spans="1:28" s="71" customFormat="1" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="64"/>
-      <c r="F38" s="83"/>
-      <c r="G38" s="83"/>
-      <c r="H38" s="83"/>
-      <c r="I38" s="84"/>
-      <c r="J38" s="84"/>
-      <c r="K38" s="64"/>
-      <c r="L38" s="64"/>
-      <c r="M38" s="99"/>
-      <c r="N38" s="99"/>
-      <c r="O38" s="84"/>
-      <c r="Q38" s="64"/>
-      <c r="R38" s="64"/>
-      <c r="S38" s="64"/>
-      <c r="T38" s="64"/>
-      <c r="U38" s="64"/>
-      <c r="V38" s="64"/>
-      <c r="X38" s="64"/>
-      <c r="Y38" s="64"/>
-      <c r="Z38" s="64"/>
-      <c r="AA38" s="64"/>
-    </row>
-    <row r="39" spans="1:28" s="88" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="86"/>
-      <c r="B39" s="87"/>
-      <c r="F39" s="89"/>
-      <c r="G39" s="89"/>
-      <c r="H39" s="89"/>
-      <c r="I39" s="90"/>
-      <c r="J39" s="90"/>
-      <c r="L39" s="86"/>
-      <c r="N39" s="89"/>
-      <c r="U39" s="86"/>
-      <c r="Z39" s="91"/>
-    </row>
-    <row r="40" spans="1:28" s="71" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="64"/>
-      <c r="B40" s="92"/>
-      <c r="E40" s="64"/>
-      <c r="F40" s="93"/>
-      <c r="G40" s="93"/>
-      <c r="H40" s="93"/>
-      <c r="I40" s="94"/>
-      <c r="J40" s="94"/>
-      <c r="K40" s="64"/>
-      <c r="L40" s="64"/>
-      <c r="N40" s="66"/>
-      <c r="O40" s="64"/>
-      <c r="Q40" s="64"/>
-      <c r="R40" s="95"/>
-      <c r="S40" s="64"/>
-      <c r="T40" s="64"/>
-      <c r="U40" s="64"/>
-      <c r="V40" s="64"/>
-      <c r="Z40" s="96"/>
-    </row>
-    <row r="41" spans="1:28" s="71" customFormat="1" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="64"/>
-      <c r="B41" s="83"/>
-      <c r="C41" s="84"/>
-      <c r="D41" s="84"/>
-      <c r="E41" s="64"/>
-      <c r="F41" s="83"/>
-      <c r="G41" s="83"/>
-      <c r="H41" s="83"/>
-      <c r="I41" s="84"/>
-      <c r="J41" s="84"/>
-      <c r="K41" s="64"/>
-      <c r="L41" s="64"/>
-      <c r="M41" s="64"/>
-      <c r="N41" s="64"/>
-      <c r="O41" s="64"/>
-      <c r="P41" s="64"/>
-      <c r="Q41" s="64"/>
-      <c r="R41" s="64"/>
-      <c r="S41" s="64"/>
-      <c r="T41" s="64"/>
-      <c r="U41" s="64"/>
-      <c r="V41" s="64"/>
-      <c r="Z41" s="96"/>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="Y28" s="4"/>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="Y29" s="4"/>
+    </row>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="Y30" s="4"/>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="Y31" s="4"/>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="E32" s="69"/>
+      <c r="F32" s="69"/>
+      <c r="G32" s="69"/>
+      <c r="H32" s="69"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="Y32" s="4"/>
+    </row>
+    <row r="33" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="T33" s="49"/>
+      <c r="Y33" s="4"/>
+    </row>
+    <row r="34" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="Y34" s="4"/>
+    </row>
+    <row r="35" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="1"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="58"/>
+      <c r="D35" s="58"/>
+      <c r="E35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="O35" s="58"/>
+      <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
+      <c r="S35"/>
+      <c r="T35"/>
+      <c r="W35" s="58"/>
+      <c r="X35"/>
+      <c r="AA35"/>
+    </row>
+    <row r="36" spans="1:28" s="61" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A36" s="59"/>
+      <c r="B36" s="60"/>
+      <c r="F36" s="62"/>
+      <c r="G36" s="62"/>
+      <c r="H36" s="62"/>
+      <c r="I36" s="63"/>
+      <c r="J36" s="63"/>
+      <c r="L36" s="59"/>
+      <c r="N36" s="62"/>
+      <c r="U36" s="59"/>
+      <c r="Z36" s="64"/>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A37" s="1"/>
+      <c r="B37" s="65"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="66"/>
+      <c r="G37" s="66"/>
+      <c r="H37" s="66"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="109"/>
+      <c r="N37" s="109"/>
+      <c r="P37"/>
+      <c r="Q37" s="1"/>
+      <c r="R37" s="4"/>
+      <c r="Z37" s="4"/>
+      <c r="AB37"/>
+    </row>
+    <row r="38" spans="1:28" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="58"/>
+      <c r="J38" s="58"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="109"/>
+      <c r="N38" s="109"/>
+      <c r="O38" s="58"/>
+      <c r="P38"/>
+      <c r="Q38" s="1"/>
+      <c r="R38" s="1"/>
+      <c r="Z38" s="1"/>
+      <c r="AB38"/>
+    </row>
+    <row r="39" spans="1:28" s="61" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="59"/>
+      <c r="B39" s="60"/>
+      <c r="F39" s="62"/>
+      <c r="G39" s="62"/>
+      <c r="H39" s="62"/>
+      <c r="I39" s="63"/>
+      <c r="J39" s="63"/>
+      <c r="L39" s="59"/>
+      <c r="N39" s="62"/>
+      <c r="U39" s="59"/>
+      <c r="Z39" s="64"/>
+    </row>
+    <row r="40" spans="1:28" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="1"/>
+      <c r="B40" s="65"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="66"/>
+      <c r="G40" s="66"/>
+      <c r="H40" s="66"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6"/>
+      <c r="L40" s="1"/>
+      <c r="M40"/>
+      <c r="N40" s="13"/>
+      <c r="P40"/>
+      <c r="Q40" s="1"/>
+      <c r="R40" s="4"/>
+      <c r="X40"/>
+      <c r="Y40"/>
+      <c r="Z40" s="67"/>
+      <c r="AA40"/>
+      <c r="AB40"/>
+    </row>
+    <row r="41" spans="1:28" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="14"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="58"/>
+      <c r="J41" s="58"/>
+      <c r="L41" s="1"/>
+      <c r="Q41" s="1"/>
+      <c r="R41" s="1"/>
+      <c r="X41"/>
+      <c r="Y41"/>
+      <c r="Z41" s="67"/>
+      <c r="AA41"/>
+      <c r="AB41"/>
     </row>
     <row r="42" spans="1:28" x14ac:dyDescent="0.2">
       <c r="I42" s="1"/>
@@ -3438,32 +3182,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="42">
-    <mergeCell ref="U23:Z23"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="I6:J7"/>
-    <mergeCell ref="J18:N18"/>
-    <mergeCell ref="J19:N19"/>
-    <mergeCell ref="J20:N20"/>
-    <mergeCell ref="J25:N25"/>
-    <mergeCell ref="J26:N26"/>
-    <mergeCell ref="J27:N27"/>
-    <mergeCell ref="J22:N22"/>
-    <mergeCell ref="J23:N23"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
     <mergeCell ref="M37:N38"/>
     <mergeCell ref="E6:F7"/>
     <mergeCell ref="H6:H7"/>
@@ -3480,23 +3198,44 @@
     <mergeCell ref="N3:R3"/>
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="D18:E18"/>
+    <mergeCell ref="J27:N27"/>
+    <mergeCell ref="J22:N22"/>
+    <mergeCell ref="J23:N23"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C6:D7"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="I6:J7"/>
+    <mergeCell ref="J18:N18"/>
+    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="J20:N20"/>
+    <mergeCell ref="J25:N25"/>
+    <mergeCell ref="J26:N26"/>
+    <mergeCell ref="U23:Z23"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:E8">
-    <cfRule type="expression" dxfId="4" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="8" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E11:I13">
-    <cfRule type="expression" dxfId="2" priority="6" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11:J13">
+  <conditionalFormatting sqref="E11:J13">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation showErrorMessage="1" sqref="W21 O38 W18 U18:U19 D26 I41:J41 C35:D35 W35 O35 D23:D24 I38:J38 C41:D41 D18:D21" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="K11:K13 I10" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
sort records in correct order
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionResults/Protocol_All_IWF-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionResults/Protocol_All_IWF-A4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionResults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C72DAC2-9DB5-4FFF-8C3B-481721D4315D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B267ACB-F923-4C05-8E39-6DB89B01BE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <definedName name="CategoryFilter">Results!#REF!</definedName>
     <definedName name="CLUB">Results!#REF!</definedName>
     <definedName name="Collet">#REF!</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="0">Results!$A$1:$CJ$100</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="0">Results!$A$1:$CE$100</definedName>
     <definedName name="demandé">Results!#REF!</definedName>
     <definedName name="dernier">Results!#REF!</definedName>
     <definedName name="essais">Results!#REF!</definedName>
@@ -48,7 +48,7 @@
     <definedName name="P.C.">Results!#REF!</definedName>
     <definedName name="PeséeGroupFilter">Results!#REF!</definedName>
     <definedName name="PRÉNOM">Results!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Results!$A:$Z</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Results!$A:$Y</definedName>
     <definedName name="progr.">Results!#REF!</definedName>
     <definedName name="requestedCJ">Results!$W:$W</definedName>
     <definedName name="StartGroupFilter">Results!#REF!</definedName>
@@ -103,7 +103,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{F0A7DC28-4FBA-4A0F-B1F3-C337DC82D113}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{3900BF51-743B-48C5-8537-BEDFCE69E4A8}">
       <text>
         <r>
           <rPr>
@@ -125,7 +125,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:if(condition="session.records.size() &gt; 0" lastCell="Y15")</t>
+          <t>jx:if(condition="session.records.size() &gt; 0" lastCell="Y16")</t>
         </r>
       </text>
     </comment>
@@ -147,17 +147,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="92">
   <si>
     <t>${l.lotNumber}</t>
   </si>
   <si>
-    <t>${l.membership}</t>
-  </si>
-  <si>
-    <t>${l.lastName}</t>
-  </si>
-  <si>
     <t>${l.firstName}</t>
   </si>
   <si>
@@ -221,9 +215,6 @@
     <t>${t.get("Results.Clean_and_Jerk")}</t>
   </si>
   <si>
-    <t>${t.get("Results.Membership")}</t>
-  </si>
-  <si>
     <t>${t.get("Results.Total")}</t>
   </si>
   <si>
@@ -236,15 +227,6 @@
     <t>${t.get("Timekeeper")}</t>
   </si>
   <si>
-    <t>${t.get("Referee1")}</t>
-  </si>
-  <si>
-    <t>${t.get("Referee2")}</t>
-  </si>
-  <si>
-    <t>${t.get("Referee3")}</t>
-  </si>
-  <si>
     <t>${group.item.category}</t>
   </si>
   <si>
@@ -323,9 +305,6 @@
     <t>${t.get("Results.max")}</t>
   </si>
   <si>
-    <t>${session != null ? t.get("Group") + " :" : ""} ${session.name}</t>
-  </si>
-  <si>
     <t xml:space="preserve">${session.marshallAsTO} ${session.marshallAsTO.federationId} </t>
   </si>
   <si>
@@ -402,6 +381,58 @@
   </si>
   <si>
     <t>${session.technicalController3AsTO != null ? t.get("TechnicalController") : ""}</t>
+  </si>
+  <si>
+    <t>${t.get("Name")}</t>
+  </si>
+  <si>
+    <t>${competition.competitionName}</t>
+  </si>
+  <si>
+    <t>${competition.competitionCity},  ${competition.competitionDate} - ${competition.competitionEndDate}</t>
+  </si>
+  <si>
+    <t>${t.get("CenterReferee")}</t>
+  </si>
+  <si>
+    <t>${t.get("SideReferee")}</t>
+  </si>
+  <si>
+    <t>${l.team}</t>
+  </si>
+  <si>
+    <t>${t.get("Team")}</t>
+  </si>
+  <si>
+    <t>${l.lastName.toUpperCase()}</t>
+  </si>
+  <si>
+    <t>${t.get("Lot")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.RecordKind")}</t>
+  </si>
+  <si>
+    <t>${r.resRecordLift}</t>
+  </si>
+  <si>
+    <t>Note: Records listed are not official until formally approved by the respective federations.  The listing is based on information available publicly at the date of the competition.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">${t.get("Group") +  session.name + " : " + " " + session.description}       </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">${session.intlStartDay +  " " + session.intlStartHour}  </t>
+    </r>
+  </si>
+  <si>
+    <t>Technical Officials</t>
   </si>
 </sst>
 </file>
@@ -414,7 +445,7 @@
     <numFmt numFmtId="166" formatCode="0;\(0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.000;;\-"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -479,11 +510,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -519,12 +545,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="9"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -573,22 +593,9 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
@@ -604,7 +611,20 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -694,7 +714,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -857,10 +877,10 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="8"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </top>
       <bottom style="thin">
         <color indexed="8"/>
@@ -872,19 +892,122 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
       <right/>
       <top style="thin">
@@ -895,20 +1018,7 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom style="thin">
         <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
       </left>
       <right/>
       <top/>
@@ -918,96 +1028,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1024,7 +1051,7 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1032,7 +1059,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1050,302 +1077,228 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="26" fillId="14" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="29" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="29" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="30" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="11" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1360,10 +1313,7 @@
     <xf numFmtId="0" fontId="9" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -1371,39 +1321,130 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="11" xfId="11" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -1875,19 +1916,20 @@
   <sheetPr codeName="Feuil4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB126"/>
+  <dimension ref="A1:Y126"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.85546875" customWidth="1"/>
-    <col min="2" max="2" width="5.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="3.140625" customWidth="1"/>
-    <col min="4" max="4" width="35.28515625" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" customWidth="1"/>
-    <col min="7" max="8" width="20.28515625" customWidth="1"/>
-    <col min="9" max="9" width="3.140625" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="3.42578125" customWidth="1"/>
     <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.28515625" style="2" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" style="1" customWidth="1"/>
     <col min="14" max="16" width="7.7109375" style="1" customWidth="1"/>
@@ -1899,321 +1941,329 @@
     <col min="23" max="23" width="7.7109375" customWidth="1"/>
     <col min="24" max="24" width="8.42578125" style="1" customWidth="1"/>
     <col min="25" max="25" width="7" style="1" customWidth="1"/>
-    <col min="26" max="26" width="7" style="3" customWidth="1"/>
-    <col min="27" max="27" width="10.140625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="8.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16"/>
-      <c r="B1" s="17"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110"/>
-      <c r="P1" s="110"/>
-      <c r="Q1" s="110"/>
-      <c r="R1" s="110"/>
-      <c r="S1" s="110"/>
-      <c r="T1" s="110"/>
-      <c r="U1" s="110"/>
-      <c r="V1" s="110"/>
-      <c r="W1" s="110"/>
-      <c r="X1" s="110"/>
-      <c r="Y1" s="110"/>
-      <c r="Z1" s="110"/>
-    </row>
-    <row r="2" spans="1:28" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="50"/>
-      <c r="O2" s="51"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="53"/>
-      <c r="R2" s="53"/>
-      <c r="S2" s="53"/>
-      <c r="T2" s="53"/>
-      <c r="U2" s="51"/>
-      <c r="V2" s="13"/>
-      <c r="X2" s="51"/>
-      <c r="Y2" s="51"/>
-    </row>
-    <row r="3" spans="1:28" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="54"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="83"/>
-      <c r="O3" s="83"/>
-      <c r="P3" s="83"/>
-      <c r="Q3" s="83"/>
-      <c r="R3" s="83"/>
-      <c r="S3" s="55"/>
-      <c r="T3" s="55"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="13"/>
-      <c r="X3" s="57"/>
-      <c r="Y3" s="57"/>
-    </row>
-    <row r="4" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="115" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="115"/>
-      <c r="C4" s="115"/>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="115"/>
-      <c r="S4" s="115"/>
-      <c r="T4" s="115"/>
-      <c r="U4" s="115"/>
-      <c r="V4" s="115"/>
-      <c r="W4" s="115"/>
-      <c r="X4" s="115"/>
-      <c r="Y4" s="115"/>
-      <c r="Z4" s="115"/>
-    </row>
-    <row r="5" spans="1:28" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="84" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="85"/>
-      <c r="C6" s="95" t="s">
+    <row r="1" spans="1:25" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="83"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="83"/>
+      <c r="T1" s="83"/>
+      <c r="U1" s="83"/>
+      <c r="V1" s="83"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+    </row>
+    <row r="2" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="123" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="123"/>
+      <c r="C2" s="123"/>
+      <c r="D2" s="123"/>
+      <c r="E2" s="123"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="123"/>
+      <c r="H2" s="123"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="123"/>
+      <c r="M2" s="123"/>
+      <c r="N2" s="123"/>
+      <c r="O2" s="123"/>
+      <c r="P2" s="123"/>
+      <c r="Q2" s="123"/>
+      <c r="R2" s="123"/>
+      <c r="S2" s="123"/>
+      <c r="T2" s="123"/>
+      <c r="U2" s="123"/>
+      <c r="V2" s="123"/>
+      <c r="W2" s="123"/>
+      <c r="X2" s="123"/>
+      <c r="Y2" s="37"/>
+    </row>
+    <row r="3" spans="1:25" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="128" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="128"/>
+      <c r="C3" s="128"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="128"/>
+      <c r="G3" s="128"/>
+      <c r="H3" s="128"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="128"/>
+      <c r="L3" s="128"/>
+      <c r="M3" s="128"/>
+      <c r="N3" s="128"/>
+      <c r="O3" s="128"/>
+      <c r="P3" s="128"/>
+      <c r="Q3" s="128"/>
+      <c r="R3" s="128"/>
+      <c r="S3" s="128"/>
+      <c r="T3" s="128"/>
+      <c r="U3" s="128"/>
+      <c r="V3" s="128"/>
+      <c r="W3" s="128"/>
+      <c r="X3" s="128"/>
+      <c r="Y3" s="40"/>
+    </row>
+    <row r="4" spans="1:25" s="53" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="124" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="124"/>
+      <c r="C4" s="124"/>
+      <c r="D4" s="124"/>
+      <c r="E4" s="124"/>
+      <c r="F4" s="124"/>
+      <c r="G4" s="124"/>
+      <c r="H4" s="124"/>
+      <c r="I4" s="124"/>
+      <c r="J4" s="124"/>
+      <c r="K4" s="124"/>
+      <c r="L4" s="124"/>
+      <c r="M4" s="124"/>
+      <c r="N4" s="124"/>
+      <c r="O4" s="124"/>
+      <c r="P4" s="124"/>
+      <c r="Q4" s="124"/>
+      <c r="R4" s="124"/>
+      <c r="S4" s="124"/>
+      <c r="T4" s="124"/>
+      <c r="U4" s="124"/>
+      <c r="V4" s="124"/>
+      <c r="W4" s="124"/>
+      <c r="X4" s="124"/>
+    </row>
+    <row r="5" spans="1:25" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="125" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="127" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="127"/>
+      <c r="D6" s="127"/>
+      <c r="E6" s="77" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="78"/>
+      <c r="G6" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="96"/>
-      <c r="E6" s="95" t="s">
+      <c r="I6" s="119" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="96"/>
-      <c r="G6" s="88" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6" s="88" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="101" t="s">
+      <c r="J6" s="120"/>
+      <c r="K6" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="102"/>
-      <c r="K6" s="88" t="s">
+      <c r="L6" s="85" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" s="86"/>
+      <c r="N6" s="86"/>
+      <c r="O6" s="86"/>
+      <c r="P6" s="86"/>
+      <c r="Q6" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="111" t="s">
+      <c r="R6" s="86"/>
+      <c r="S6" s="86"/>
+      <c r="T6" s="86"/>
+      <c r="U6" s="86"/>
+      <c r="V6" s="86"/>
+      <c r="W6" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="112"/>
-      <c r="N6" s="112"/>
-      <c r="O6" s="112"/>
-      <c r="P6" s="112"/>
-      <c r="Q6" s="111" t="s">
+      <c r="X6" s="88"/>
+      <c r="Y6" s="84"/>
+    </row>
+    <row r="7" spans="1:25" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="126"/>
+      <c r="B7" s="127"/>
+      <c r="C7" s="127"/>
+      <c r="D7" s="127"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="80"/>
+      <c r="G7" s="82"/>
+      <c r="H7" s="82"/>
+      <c r="I7" s="121"/>
+      <c r="J7" s="122"/>
+      <c r="K7" s="82"/>
+      <c r="L7" s="30">
+        <v>1</v>
+      </c>
+      <c r="M7" s="31">
+        <v>2</v>
+      </c>
+      <c r="N7" s="31">
+        <v>3</v>
+      </c>
+      <c r="O7" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="P7" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="112"/>
-      <c r="S6" s="112"/>
-      <c r="T6" s="112"/>
-      <c r="U6" s="112"/>
-      <c r="V6" s="112"/>
-      <c r="W6" s="113" t="s">
-        <v>25</v>
-      </c>
-      <c r="X6" s="114"/>
-      <c r="Y6" s="122"/>
-      <c r="Z6" s="122"/>
-      <c r="AB6"/>
-    </row>
-    <row r="7" spans="1:28" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="84"/>
-      <c r="B7" s="85"/>
-      <c r="C7" s="97"/>
-      <c r="D7" s="98"/>
-      <c r="E7" s="97"/>
-      <c r="F7" s="98"/>
-      <c r="G7" s="89"/>
-      <c r="H7" s="89"/>
-      <c r="I7" s="103"/>
-      <c r="J7" s="104"/>
-      <c r="K7" s="89"/>
-      <c r="L7" s="42">
+      <c r="Q7" s="31">
         <v>1</v>
       </c>
-      <c r="M7" s="43">
+      <c r="R7" s="31">
         <v>2</v>
       </c>
-      <c r="N7" s="43">
+      <c r="S7" s="89">
         <v>3</v>
       </c>
-      <c r="O7" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="P7" s="45" t="s">
+      <c r="T7" s="90"/>
+      <c r="U7" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="V7" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="W7" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="X7" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y7" s="84"/>
+    </row>
+    <row r="8" spans="1:25" s="10" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="18"/>
+    </row>
+    <row r="9" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="Q7" s="43">
+      <c r="B9" s="20"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="21"/>
+      <c r="O9" s="21"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21"/>
+      <c r="T9" s="21"/>
+      <c r="U9" s="21"/>
+      <c r="V9" s="21"/>
+      <c r="W9" s="21"/>
+      <c r="X9" s="52"/>
+      <c r="Y9" s="51"/>
+    </row>
+    <row r="10" spans="1:25" s="10" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="104" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="104"/>
+      <c r="D10" s="104"/>
+      <c r="E10" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="R7" s="43">
+      <c r="F10" s="94"/>
+      <c r="G10" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="H10" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="S7" s="116">
+      <c r="I10" s="110" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" s="111"/>
+      <c r="K10" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="N10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="O10" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="P10" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q10" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="R10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="S10" s="91" t="s">
+        <v>11</v>
+      </c>
+      <c r="T10" s="92"/>
+      <c r="U10" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="V10" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="W10" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="T7" s="117"/>
-      <c r="U7" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="V7" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="W7" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="X7" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y7" s="122"/>
-      <c r="Z7" s="122"/>
-    </row>
-    <row r="8" spans="1:28" s="11" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="20"/>
-      <c r="Y8" s="123"/>
-      <c r="Z8" s="123"/>
-    </row>
-    <row r="9" spans="1:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="23"/>
-      <c r="S9" s="23"/>
-      <c r="T9" s="23"/>
-      <c r="U9" s="23"/>
-      <c r="V9" s="23"/>
-      <c r="W9" s="23"/>
-      <c r="X9" s="127"/>
-      <c r="Y9" s="125"/>
-      <c r="Z9" s="126"/>
-      <c r="AB9"/>
-    </row>
-    <row r="10" spans="1:28" s="11" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="36"/>
-      <c r="E10" s="120" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="121"/>
-      <c r="G10" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="I10" s="99" t="s">
-        <v>14</v>
-      </c>
-      <c r="J10" s="100"/>
-      <c r="K10" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="M10" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="N10" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="O10" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="P10" s="39" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="R10" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="S10" s="118" t="s">
-        <v>13</v>
-      </c>
-      <c r="T10" s="119"/>
-      <c r="U10" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="V10" s="39" t="s">
-        <v>55</v>
-      </c>
-      <c r="W10" s="40" t="s">
-        <v>5</v>
-      </c>
-      <c r="X10" s="41" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y10" s="124"/>
-      <c r="Z10" s="124"/>
-    </row>
-    <row r="11" spans="1:28" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X10" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y10" s="50"/>
+    </row>
+    <row r="11" spans="1:25" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11"/>
       <c r="K11"/>
       <c r="L11"/>
@@ -2227,643 +2277,626 @@
       <c r="V11"/>
       <c r="X11"/>
       <c r="Y11"/>
-      <c r="Z11"/>
-      <c r="AA11"/>
-      <c r="AB11"/>
-    </row>
-    <row r="12" spans="1:28" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    </row>
+    <row r="12" spans="1:25" s="74" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="74" t="s">
+        <v>33</v>
+      </c>
+      <c r="M12" s="55"/>
+    </row>
+    <row r="13" spans="1:25" s="14" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="22"/>
+      <c r="Q13" s="22"/>
+      <c r="R13" s="22"/>
+      <c r="S13" s="23"/>
+      <c r="T13" s="23"/>
+      <c r="U13" s="23"/>
+      <c r="V13" s="23"/>
+      <c r="W13" s="23"/>
+      <c r="X13" s="23"/>
+      <c r="Y13" s="23"/>
+    </row>
+    <row r="14" spans="1:25" s="14" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="97" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="98"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="63" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="97" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="99"/>
+      <c r="G14" s="63" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="97" t="s">
+        <v>87</v>
+      </c>
+      <c r="J14" s="98"/>
+      <c r="K14" s="97" t="s">
+        <v>35</v>
+      </c>
+      <c r="L14" s="98"/>
+      <c r="M14" s="103" t="s">
+        <v>78</v>
+      </c>
+      <c r="N14" s="103"/>
+      <c r="O14" s="103"/>
+      <c r="P14" s="103"/>
+      <c r="Q14" s="103"/>
+      <c r="R14" s="103"/>
+      <c r="S14" s="97" t="s">
+        <v>18</v>
+      </c>
+      <c r="T14" s="98"/>
+      <c r="U14" s="99"/>
+      <c r="V14" s="97" t="s">
+        <v>19</v>
+      </c>
+      <c r="W14" s="98"/>
+      <c r="X14" s="99"/>
+      <c r="Y14" s="64"/>
+    </row>
+    <row r="15" spans="1:25" s="72" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="112" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="113"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="65" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="115" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="116"/>
+      <c r="G15" s="66" t="s">
+        <v>40</v>
+      </c>
+      <c r="H15" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="M12" s="17"/>
-    </row>
-    <row r="13" spans="1:28" s="16" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="25"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="28"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="25"/>
-      <c r="R13" s="25"/>
-      <c r="S13" s="28"/>
-      <c r="T13" s="28"/>
-      <c r="U13" s="28"/>
-      <c r="V13" s="28"/>
-      <c r="W13" s="28"/>
-      <c r="X13" s="28"/>
-      <c r="Y13" s="28"/>
-      <c r="Z13" s="28"/>
-    </row>
-    <row r="14" spans="1:28" s="33" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="92" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="93"/>
-      <c r="C14" s="94"/>
-      <c r="D14" s="71" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" s="92" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="94"/>
-      <c r="G14" s="71" t="s">
-        <v>43</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="I14" s="92" t="s">
+      <c r="I15" s="108" t="s">
+        <v>88</v>
+      </c>
+      <c r="J15" s="109"/>
+      <c r="K15" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="L15" s="118"/>
+      <c r="M15" s="100" t="s">
         <v>41</v>
       </c>
-      <c r="J14" s="93"/>
-      <c r="K14" s="76" t="s">
-        <v>41</v>
-      </c>
-      <c r="L14" s="76"/>
-      <c r="M14" s="76"/>
-      <c r="N14" s="76"/>
-      <c r="O14" s="76"/>
-      <c r="P14" s="30"/>
-      <c r="Q14" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="R14" s="29"/>
-      <c r="S14" s="32"/>
-      <c r="T14" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="U14" s="76"/>
-      <c r="V14" s="30"/>
-      <c r="W14" s="81"/>
-      <c r="Y14" s="81"/>
-      <c r="AB14" s="30"/>
-    </row>
-    <row r="15" spans="1:28" s="24" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="106" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="107"/>
-      <c r="C15" s="108"/>
-      <c r="D15" s="73" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="86" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" s="87"/>
-      <c r="G15" s="75" t="s">
-        <v>46</v>
-      </c>
-      <c r="H15" s="72" t="s">
-        <v>45</v>
-      </c>
-      <c r="I15" s="90" t="s">
-        <v>35</v>
-      </c>
-      <c r="J15" s="91"/>
-      <c r="K15" s="74" t="s">
-        <v>47</v>
-      </c>
-      <c r="L15" s="74" t="s">
-        <v>47</v>
-      </c>
-      <c r="M15" s="79"/>
-      <c r="N15" s="79"/>
-      <c r="O15" s="79"/>
-      <c r="P15" s="80"/>
-      <c r="Q15" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="R15" s="27"/>
-      <c r="S15" s="26"/>
-      <c r="T15" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="U15" s="78"/>
-      <c r="V15" s="26"/>
-      <c r="W15" s="82"/>
-      <c r="Y15" s="82"/>
-      <c r="AB15" s="26"/>
-    </row>
-    <row r="16" spans="1:28" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="6"/>
+      <c r="N15" s="101"/>
+      <c r="O15" s="101"/>
+      <c r="P15" s="101"/>
+      <c r="Q15" s="101"/>
+      <c r="R15" s="102"/>
+      <c r="S15" s="105" t="s">
+        <v>30</v>
+      </c>
+      <c r="T15" s="106"/>
+      <c r="U15" s="107"/>
+      <c r="V15" s="69" t="s">
+        <v>32</v>
+      </c>
+      <c r="W15" s="70"/>
+      <c r="X15" s="68"/>
+      <c r="Y15" s="71"/>
+    </row>
+    <row r="16" spans="1:25" s="5" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="75" t="s">
+        <v>89</v>
+      </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
       <c r="K16" s="7"/>
       <c r="L16" s="6"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
       <c r="O16" s="6"/>
       <c r="Q16" s="8"/>
       <c r="S16" s="6"/>
       <c r="T16" s="6"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="15"/>
-      <c r="W16" s="15"/>
+      <c r="U16" s="13"/>
+      <c r="V16" s="13"/>
+      <c r="W16" s="13"/>
       <c r="X16" s="6"/>
       <c r="Y16" s="4"/>
-      <c r="Z16" s="8"/>
-      <c r="AA16" s="6"/>
-      <c r="AB16" s="6"/>
-    </row>
-    <row r="17" spans="1:28" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="C17" s="6"/>
+    </row>
+    <row r="17" spans="1:25" s="5" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="74" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="74"/>
+      <c r="C17" s="74"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
       <c r="K17" s="7"/>
       <c r="L17" s="6"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
       <c r="O17" s="6"/>
       <c r="Q17" s="8"/>
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
-      <c r="U17" s="15"/>
-      <c r="V17" s="15"/>
-      <c r="W17" s="15"/>
+      <c r="U17" s="13"/>
+      <c r="V17" s="13"/>
+      <c r="W17" s="13"/>
       <c r="X17" s="6"/>
       <c r="Y17" s="4"/>
-      <c r="Z17" s="8"/>
-      <c r="AA17" s="6"/>
-      <c r="AB17" s="6"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B18" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D18" s="83" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="83"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="60" t="s">
-        <v>83</v>
-      </c>
-      <c r="J18" s="105" t="s">
+    </row>
+    <row r="18" spans="1:25" s="35" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="56" t="s">
+        <v>81</v>
+      </c>
+      <c r="D18" s="95" t="s">
+        <v>43</v>
+      </c>
+      <c r="E18" s="95"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="56" t="s">
+        <v>76</v>
+      </c>
+      <c r="J18" s="96" t="s">
+        <v>59</v>
+      </c>
+      <c r="K18" s="96"/>
+      <c r="L18" s="96"/>
+      <c r="M18" s="96"/>
+      <c r="N18" s="96"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="56" t="s">
+        <v>70</v>
+      </c>
+      <c r="U18" s="58" t="s">
+        <v>46</v>
+      </c>
+      <c r="V18" s="59"/>
+      <c r="W18" s="58"/>
+      <c r="Y18" s="39"/>
+    </row>
+    <row r="19" spans="1:25" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B19" s="56" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19" s="95" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19" s="95"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="56" t="s">
+        <v>76</v>
+      </c>
+      <c r="J19" s="96" t="s">
+        <v>60</v>
+      </c>
+      <c r="K19" s="96"/>
+      <c r="L19" s="96"/>
+      <c r="M19" s="96"/>
+      <c r="N19" s="96"/>
+      <c r="S19" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="T19" s="56"/>
+      <c r="U19" s="58" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B20" s="56" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="95" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="95"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
+      <c r="H20" s="56" t="s">
+        <v>77</v>
+      </c>
+      <c r="J20" s="96" t="s">
+        <v>61</v>
+      </c>
+      <c r="K20" s="96"/>
+      <c r="L20" s="96"/>
+      <c r="M20" s="96"/>
+      <c r="N20" s="96"/>
+      <c r="R20" s="14"/>
+      <c r="S20" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="T20" s="39"/>
+      <c r="U20" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="V20" s="56"/>
+      <c r="W20" s="39"/>
+      <c r="Y20" s="39"/>
+    </row>
+    <row r="21" spans="1:25" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B21" s="56" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="95" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="95"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="56"/>
+      <c r="J21" s="38"/>
+      <c r="K21" s="38"/>
+      <c r="L21" s="38"/>
+      <c r="M21" s="38"/>
+      <c r="R21" s="14"/>
+      <c r="S21" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="T21" s="39"/>
+      <c r="U21" s="58" t="s">
+        <v>56</v>
+      </c>
+      <c r="V21" s="56"/>
+      <c r="W21" s="58"/>
+      <c r="Y21" s="39"/>
+    </row>
+    <row r="22" spans="1:25" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B22" s="56"/>
+      <c r="D22" s="61"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="56" t="s">
+        <v>69</v>
+      </c>
+      <c r="J22" s="96" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="105"/>
-      <c r="L18" s="105"/>
-      <c r="M18" s="105"/>
-      <c r="N18" s="105"/>
-      <c r="O18"/>
-      <c r="P18"/>
-      <c r="R18" s="5"/>
-      <c r="S18" s="60" t="s">
-        <v>77</v>
-      </c>
-      <c r="T18"/>
-      <c r="U18" s="58" t="s">
+      <c r="K22" s="96"/>
+      <c r="L22" s="96"/>
+      <c r="M22" s="96"/>
+      <c r="N22" s="96"/>
+      <c r="S22" s="56" t="s">
+        <v>65</v>
+      </c>
+      <c r="U22" s="58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B23" s="56" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="95" t="s">
         <v>52</v>
       </c>
-      <c r="V18" s="15"/>
-      <c r="W18" s="58"/>
-      <c r="X18"/>
-      <c r="AA18"/>
-    </row>
-    <row r="19" spans="1:28" s="61" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="83" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="83"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="60" t="s">
-        <v>83</v>
-      </c>
-      <c r="J19" s="105" t="s">
+      <c r="E23" s="95"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="56" t="s">
+        <v>69</v>
+      </c>
+      <c r="J23" s="96" t="s">
+        <v>68</v>
+      </c>
+      <c r="K23" s="96"/>
+      <c r="L23" s="96"/>
+      <c r="M23" s="96"/>
+      <c r="N23" s="96"/>
+      <c r="R23" s="14"/>
+      <c r="S23" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="K19" s="105"/>
-      <c r="L19" s="105"/>
-      <c r="M19" s="105"/>
-      <c r="N19" s="105"/>
-      <c r="S19" s="60" t="s">
+      <c r="T23" s="39"/>
+      <c r="U23" s="95" t="s">
+        <v>58</v>
+      </c>
+      <c r="V23" s="95"/>
+      <c r="W23" s="95"/>
+      <c r="X23" s="95"/>
+      <c r="Y23" s="95"/>
+    </row>
+    <row r="24" spans="1:25" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B24" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="95" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="95"/>
+      <c r="H24" s="14"/>
+      <c r="S24" s="39"/>
+      <c r="T24" s="39"/>
+      <c r="U24" s="39"/>
+      <c r="V24" s="39"/>
+    </row>
+    <row r="25" spans="1:25" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="D25" s="61"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="56" t="s">
+        <v>71</v>
+      </c>
+      <c r="J25" s="96" t="s">
+        <v>62</v>
+      </c>
+      <c r="K25" s="96"/>
+      <c r="L25" s="96"/>
+      <c r="M25" s="96"/>
+      <c r="N25" s="96"/>
+      <c r="O25" s="15"/>
+      <c r="V25" s="15"/>
+      <c r="W25" s="15"/>
+    </row>
+    <row r="26" spans="1:25" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B26" s="56" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="95" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" s="95"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="56" t="s">
         <v>72</v>
       </c>
-      <c r="T19" s="60"/>
-      <c r="U19" s="58" t="s">
-        <v>61</v>
-      </c>
-      <c r="Z19" s="64"/>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B20" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="83" t="s">
-        <v>50</v>
-      </c>
-      <c r="E20" s="83"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="60" t="s">
-        <v>84</v>
-      </c>
-      <c r="J20" s="105" t="s">
-        <v>68</v>
-      </c>
-      <c r="K20" s="105"/>
-      <c r="L20" s="105"/>
-      <c r="M20" s="105"/>
-      <c r="N20" s="105"/>
-      <c r="O20"/>
-      <c r="P20"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="60" t="s">
-        <v>72</v>
-      </c>
-      <c r="U20" s="58" t="s">
-        <v>62</v>
-      </c>
-      <c r="V20" s="14"/>
-      <c r="W20" s="1"/>
-      <c r="X20"/>
-      <c r="Z20" s="4"/>
-      <c r="AB20"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B21" s="60" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="83"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="65"/>
-      <c r="J21" s="68"/>
-      <c r="K21" s="68"/>
-      <c r="L21" s="68"/>
-      <c r="M21" s="68"/>
-      <c r="N21"/>
-      <c r="O21"/>
-      <c r="P21"/>
-      <c r="R21" s="5"/>
-      <c r="S21" s="60" t="s">
-        <v>72</v>
-      </c>
-      <c r="U21" s="58" t="s">
+      <c r="J26" s="96" t="s">
         <v>63</v>
       </c>
-      <c r="V21" s="14"/>
-      <c r="W21" s="58"/>
-      <c r="X21"/>
-      <c r="Z21" s="1"/>
-      <c r="AB21"/>
-    </row>
-    <row r="22" spans="1:28" s="61" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="14"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="70"/>
-      <c r="G22" s="70"/>
-      <c r="H22" s="60" t="s">
-        <v>76</v>
-      </c>
-      <c r="J22" s="105" t="s">
+      <c r="K26" s="96"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="96"/>
+      <c r="N26" s="96"/>
+      <c r="O26" s="39"/>
+      <c r="Q26" s="54"/>
+      <c r="R26" s="39"/>
+      <c r="S26" s="39"/>
+      <c r="T26" s="39"/>
+      <c r="U26" s="39"/>
+      <c r="W26" s="39"/>
+      <c r="X26" s="60"/>
+      <c r="Y26" s="39"/>
+    </row>
+    <row r="27" spans="1:25" s="35" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="B27" s="39"/>
+      <c r="F27" s="57"/>
+      <c r="G27" s="57"/>
+      <c r="H27" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="K22" s="105"/>
-      <c r="L22" s="105"/>
-      <c r="M22" s="105"/>
-      <c r="N22" s="105"/>
-      <c r="S22" s="60" t="s">
-        <v>72</v>
-      </c>
-      <c r="U22" s="58" t="s">
+      <c r="J27" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="Z22" s="64"/>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B23" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="83" t="s">
-        <v>59</v>
-      </c>
-      <c r="E23" s="83"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
-      <c r="H23" s="60" t="s">
-        <v>76</v>
-      </c>
-      <c r="J23" s="105" t="s">
-        <v>75</v>
-      </c>
-      <c r="K23" s="105"/>
-      <c r="L23" s="105"/>
-      <c r="M23" s="105"/>
-      <c r="N23" s="105"/>
-      <c r="O23"/>
-      <c r="P23"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="60" t="s">
-        <v>74</v>
-      </c>
-      <c r="U23" s="83" t="s">
-        <v>65</v>
-      </c>
-      <c r="V23" s="83"/>
-      <c r="W23" s="83"/>
-      <c r="X23" s="83"/>
-      <c r="Y23" s="83"/>
-      <c r="Z23" s="83"/>
-      <c r="AA23"/>
-      <c r="AB23"/>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B24" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D24" s="83" t="s">
-        <v>60</v>
-      </c>
-      <c r="E24" s="83"/>
-      <c r="H24" s="5"/>
-      <c r="K24"/>
-      <c r="L24"/>
-      <c r="M24"/>
-      <c r="N24"/>
-      <c r="O24"/>
-      <c r="P24"/>
-      <c r="R24"/>
-      <c r="X24"/>
-      <c r="Y24"/>
-      <c r="Z24" s="67"/>
-      <c r="AA24"/>
-      <c r="AB24"/>
-    </row>
-    <row r="25" spans="1:28" s="61" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D25" s="63"/>
-      <c r="E25" s="59"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="60" t="s">
-        <v>78</v>
-      </c>
-      <c r="J25" s="105" t="s">
-        <v>69</v>
-      </c>
-      <c r="K25" s="105"/>
-      <c r="L25" s="105"/>
-      <c r="M25" s="105"/>
-      <c r="N25" s="105"/>
-      <c r="O25" s="59"/>
-      <c r="V25" s="59"/>
-      <c r="W25" s="59"/>
-      <c r="Z25" s="64"/>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B26" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="83" t="s">
-        <v>51</v>
-      </c>
-      <c r="E26" s="83"/>
-      <c r="F26" s="70"/>
-      <c r="G26" s="70"/>
-      <c r="H26" s="60" t="s">
-        <v>79</v>
-      </c>
-      <c r="J26" s="105" t="s">
-        <v>70</v>
-      </c>
-      <c r="K26" s="105"/>
-      <c r="L26" s="105"/>
-      <c r="M26" s="105"/>
-      <c r="N26" s="105"/>
-      <c r="P26"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="1"/>
-      <c r="V26"/>
-      <c r="W26" s="1"/>
-      <c r="X26" s="4"/>
-    </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="J27" s="105" t="s">
-        <v>71</v>
-      </c>
-      <c r="K27" s="105"/>
-      <c r="L27" s="105"/>
-      <c r="M27" s="105"/>
-      <c r="N27" s="105"/>
-      <c r="Y27" s="4"/>
-    </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-      <c r="Y28" s="4"/>
-    </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="K27" s="96"/>
+      <c r="L27" s="96"/>
+      <c r="M27" s="96"/>
+      <c r="N27" s="96"/>
+      <c r="O27" s="39"/>
+      <c r="P27" s="39"/>
+      <c r="R27" s="54"/>
+      <c r="S27" s="39"/>
+      <c r="T27" s="39"/>
+      <c r="U27" s="39"/>
+      <c r="V27" s="39"/>
+      <c r="X27" s="39"/>
+      <c r="Y27" s="60"/>
+    </row>
+    <row r="28" spans="1:25" s="35" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B28" s="39"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="39"/>
+      <c r="K28" s="39"/>
+      <c r="L28" s="39"/>
+      <c r="M28" s="39"/>
+      <c r="N28" s="39"/>
+      <c r="O28" s="39"/>
+      <c r="P28" s="39"/>
+      <c r="R28" s="54"/>
+      <c r="S28" s="39"/>
+      <c r="T28" s="39"/>
+      <c r="U28" s="39"/>
+      <c r="V28" s="39"/>
+      <c r="X28" s="39"/>
+      <c r="Y28" s="60"/>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="Y29" s="4"/>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="Y30" s="4"/>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="Y31" s="4"/>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="E32" s="69"/>
-      <c r="F32" s="69"/>
-      <c r="G32" s="69"/>
-      <c r="H32" s="69"/>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="Y32" s="4"/>
     </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
-      <c r="T33" s="49"/>
+      <c r="T33" s="36"/>
       <c r="Y33" s="4"/>
     </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="Y34" s="4"/>
     </row>
-    <row r="35" spans="1:28" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="58"/>
-      <c r="D35" s="58"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
       <c r="E35" s="1"/>
       <c r="L35" s="1"/>
-      <c r="O35" s="58"/>
+      <c r="O35" s="41"/>
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
       <c r="S35"/>
       <c r="T35"/>
-      <c r="W35" s="58"/>
+      <c r="W35" s="41"/>
       <c r="X35"/>
-      <c r="AA35"/>
-    </row>
-    <row r="36" spans="1:28" s="61" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A36" s="59"/>
-      <c r="B36" s="60"/>
-      <c r="F36" s="62"/>
-      <c r="G36" s="62"/>
-      <c r="H36" s="62"/>
-      <c r="I36" s="63"/>
-      <c r="J36" s="63"/>
-      <c r="L36" s="59"/>
-      <c r="N36" s="62"/>
-      <c r="U36" s="59"/>
-      <c r="Z36" s="64"/>
-    </row>
-    <row r="37" spans="1:28" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:25" s="44" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A36" s="42"/>
+      <c r="B36" s="43"/>
+      <c r="F36" s="45"/>
+      <c r="G36" s="45"/>
+      <c r="H36" s="45"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="46"/>
+      <c r="L36" s="42"/>
+      <c r="N36" s="45"/>
+      <c r="U36" s="42"/>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
-      <c r="B37" s="65"/>
+      <c r="B37" s="47"/>
       <c r="E37" s="1"/>
-      <c r="F37" s="66"/>
-      <c r="G37" s="66"/>
-      <c r="H37" s="66"/>
+      <c r="F37" s="48"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="48"/>
       <c r="I37" s="6"/>
       <c r="J37" s="6"/>
       <c r="L37" s="1"/>
-      <c r="M37" s="109"/>
-      <c r="N37" s="109"/>
+      <c r="M37" s="76"/>
+      <c r="N37" s="76"/>
       <c r="P37"/>
       <c r="Q37" s="1"/>
       <c r="R37" s="4"/>
-      <c r="Z37" s="4"/>
-      <c r="AB37"/>
-    </row>
-    <row r="38" spans="1:28" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="58"/>
-      <c r="J38" s="58"/>
+    </row>
+    <row r="38" spans="1:25" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="41"/>
+      <c r="J38" s="41"/>
       <c r="L38" s="1"/>
-      <c r="M38" s="109"/>
-      <c r="N38" s="109"/>
-      <c r="O38" s="58"/>
+      <c r="M38" s="76"/>
+      <c r="N38" s="76"/>
+      <c r="O38" s="41"/>
       <c r="P38"/>
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
-      <c r="Z38" s="1"/>
-      <c r="AB38"/>
-    </row>
-    <row r="39" spans="1:28" s="61" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="59"/>
-      <c r="B39" s="60"/>
-      <c r="F39" s="62"/>
-      <c r="G39" s="62"/>
-      <c r="H39" s="62"/>
-      <c r="I39" s="63"/>
-      <c r="J39" s="63"/>
-      <c r="L39" s="59"/>
-      <c r="N39" s="62"/>
-      <c r="U39" s="59"/>
-      <c r="Z39" s="64"/>
-    </row>
-    <row r="40" spans="1:28" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="1:25" s="44" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="42"/>
+      <c r="B39" s="43"/>
+      <c r="F39" s="45"/>
+      <c r="G39" s="45"/>
+      <c r="H39" s="45"/>
+      <c r="I39" s="46"/>
+      <c r="J39" s="46"/>
+      <c r="L39" s="42"/>
+      <c r="N39" s="45"/>
+      <c r="U39" s="42"/>
+    </row>
+    <row r="40" spans="1:25" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
-      <c r="B40" s="65"/>
+      <c r="B40" s="47"/>
       <c r="E40" s="1"/>
-      <c r="F40" s="66"/>
-      <c r="G40" s="66"/>
-      <c r="H40" s="66"/>
+      <c r="F40" s="48"/>
+      <c r="G40" s="48"/>
+      <c r="H40" s="48"/>
       <c r="I40" s="6"/>
       <c r="J40" s="6"/>
       <c r="L40" s="1"/>
       <c r="M40"/>
-      <c r="N40" s="13"/>
+      <c r="N40" s="11"/>
       <c r="P40"/>
       <c r="Q40" s="1"/>
       <c r="R40" s="4"/>
       <c r="X40"/>
       <c r="Y40"/>
-      <c r="Z40" s="67"/>
-      <c r="AA40"/>
-      <c r="AB40"/>
-    </row>
-    <row r="41" spans="1:28" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:25" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="58"/>
-      <c r="D41" s="58"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
       <c r="E41" s="1"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="58"/>
-      <c r="J41" s="58"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="41"/>
+      <c r="J41" s="41"/>
       <c r="L41" s="1"/>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
       <c r="X41"/>
       <c r="Y41"/>
-      <c r="Z41" s="67"/>
-      <c r="AA41"/>
-      <c r="AB41"/>
-    </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
     </row>
-    <row r="43" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
     </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
     </row>
-    <row r="45" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
     </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
     </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I47" s="1"/>
       <c r="J47" s="1"/>
     </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.2">
       <c r="I48" s="1"/>
       <c r="J48" s="1"/>
     </row>
@@ -3181,49 +3214,57 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="42">
+  <mergeCells count="50">
+    <mergeCell ref="A2:X2"/>
+    <mergeCell ref="A3:X3"/>
+    <mergeCell ref="A4:X4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:D7"/>
+    <mergeCell ref="U23:Y23"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="I6:J7"/>
+    <mergeCell ref="J18:N18"/>
+    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="M15:R15"/>
+    <mergeCell ref="M14:R14"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="V14:X14"/>
+    <mergeCell ref="S14:U14"/>
+    <mergeCell ref="S15:U15"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="J20:N20"/>
+    <mergeCell ref="J25:N25"/>
+    <mergeCell ref="J26:N26"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D23:E23"/>
     <mergeCell ref="M37:N38"/>
     <mergeCell ref="E6:F7"/>
     <mergeCell ref="H6:H7"/>
-    <mergeCell ref="N1:Z1"/>
-    <mergeCell ref="Y6:Z7"/>
-    <mergeCell ref="Y10:Z10"/>
+    <mergeCell ref="N1:Y1"/>
+    <mergeCell ref="Y6:Y7"/>
     <mergeCell ref="L6:P6"/>
     <mergeCell ref="Q6:V6"/>
     <mergeCell ref="W6:X6"/>
-    <mergeCell ref="A4:Z4"/>
     <mergeCell ref="S7:T7"/>
     <mergeCell ref="S10:T10"/>
     <mergeCell ref="E10:F10"/>
-    <mergeCell ref="N3:R3"/>
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="J27:N27"/>
     <mergeCell ref="J22:N22"/>
     <mergeCell ref="J23:N23"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="I6:J7"/>
-    <mergeCell ref="J18:N18"/>
-    <mergeCell ref="J19:N19"/>
-    <mergeCell ref="J20:N20"/>
-    <mergeCell ref="J25:N25"/>
-    <mergeCell ref="J26:N26"/>
-    <mergeCell ref="U23:Z23"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:E8">
     <cfRule type="expression" dxfId="1" priority="8" stopIfTrue="1">
@@ -3247,7 +3288,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.31496062992125984" right="0.35433070866141736" top="0.39370078740157483" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="70" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="57" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>